<commit_message>
WorkoutPlan OK and PhysicalAssessmentForm -> Version 1.0 Implemented
</commit_message>
<xml_diff>
--- a/WorkoutPlan.xlsx
+++ b/WorkoutPlan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0_ARTES\_Mikael\_TEMPORÁRIOS\_P\_MKR\WorkoutPlan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E079AA-8B8F-4E5A-93C2-A094033B0159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9393DFB9-EF9C-4785-A529-62F6FC846530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="64">
   <si>
     <t>Exercício</t>
   </si>
@@ -207,15 +207,6 @@
     <t>3-0-1-0</t>
   </si>
   <si>
-    <t>Supersérie (Antag.)</t>
-  </si>
-  <si>
-    <t>Supersérie (Agon.)</t>
-  </si>
-  <si>
-    <t>TUT/Cadência</t>
-  </si>
-  <si>
     <t>2-0-2-0</t>
   </si>
   <si>
@@ -234,15 +225,6 @@
     <t>4-3-2-0</t>
   </si>
   <si>
-    <t>Rep. Parciais</t>
-  </si>
-  <si>
-    <t>Pirâmide Cresc.</t>
-  </si>
-  <si>
-    <t>Pirâmide Decresc.</t>
-  </si>
-  <si>
     <t>4-0-0-0</t>
   </si>
   <si>
@@ -252,12 +234,6 @@
     <t>3-0-0-0</t>
   </si>
   <si>
-    <t>Rep. Forçadas</t>
-  </si>
-  <si>
-    <t>Rep. Roubadas</t>
-  </si>
-  <si>
     <t>5-0-5-0</t>
   </si>
   <si>
@@ -268,9 +244,6 @@
   </si>
   <si>
     <t>6-0-6-0</t>
-  </si>
-  <si>
-    <t>EMOM / AMRAP</t>
   </si>
   <si>
     <t>EMOM (Every Minute on the Minute)</t>
@@ -290,9 +263,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="171" formatCode="0&quot;s&quot;"/>
-    <numFmt numFmtId="174" formatCode="0\ &quot;min&quot;"/>
-    <numFmt numFmtId="181" formatCode="[h]&quot;h&quot;mm&quot;min&quot;"/>
+    <numFmt numFmtId="164" formatCode="0&quot;s&quot;"/>
+    <numFmt numFmtId="165" formatCode="0\ &quot;min&quot;"/>
+    <numFmt numFmtId="166" formatCode="[h]&quot;h&quot;mm&quot;min&quot;"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -377,45 +350,36 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <numFmt numFmtId="181" formatCode="[h]&quot;h&quot;mm&quot;min&quot;"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="171" formatCode="0&quot;s&quot;"/>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="171" formatCode="0&quot;s&quot;"/>
+      <numFmt numFmtId="164" formatCode="0&quot;s&quot;"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="171" formatCode="0&quot;s&quot;"/>
+      <numFmt numFmtId="164" formatCode="0&quot;s&quot;"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="171" formatCode="0&quot;s&quot;"/>
+      <numFmt numFmtId="164" formatCode="0&quot;s&quot;"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="171" formatCode="0&quot;s&quot;"/>
+      <numFmt numFmtId="164" formatCode="0&quot;s&quot;"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -587,6 +551,18 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="[h]&quot;h&quot;mm&quot;min&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0&quot;s&quot;"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -606,16 +582,16 @@
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{2B75D1C7-4FBD-44EF-8D4F-38CA297A6E5A}" name="Exercício"/>
     <tableColumn id="2" xr3:uid="{A451B7CA-E273-431C-92A1-EB5CBBAAB317}" name="Método"/>
-    <tableColumn id="3" xr3:uid="{A98EA25C-9149-40FA-8B9A-2045C7A3A6EC}" name="Séries" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{A98EA25C-9149-40FA-8B9A-2045C7A3A6EC}" name="Séries" dataDxfId="15"/>
     <tableColumn id="4" xr3:uid="{BA4AD275-29DB-444E-8F70-A82E64EE8FA8}" name="Repetições"/>
     <tableColumn id="5" xr3:uid="{84D88480-01B6-404E-BD00-7AA69D243C48}" name="Objetivo"/>
-    <tableColumn id="6" xr3:uid="{A324CD21-2CEF-4576-8F0F-CB364570E9AA}" name="Cadência (TUT)" dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{A324CD21-2CEF-4576-8F0F-CB364570E9AA}" name="Cadência (TUT)" dataDxfId="14">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(Tabela1[[#This Row],[Método]], Tabela7[Métodos/Objetivos], OFFSET(Tabela7[Métodos/Objetivos], 0, MATCH(Tabela1[[#This Row],[Objetivo]], Tabela7[#Headers], 0)-1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{84416A90-29A6-4D89-BCB3-DC3548F7118D}" name="Descanso" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{84416A90-29A6-4D89-BCB3-DC3548F7118D}" name="Descanso" dataDxfId="13">
       <calculatedColumnFormula array="1">_xlfn.XLOOKUP(Tabela1[[#This Row],[Método]], Tabela8[Métodos/Objetivos], OFFSET(Tabela8[Métodos/Objetivos], 0, MATCH(Tabela1[[#This Row],[Objetivo]], Tabela8[#Headers], 0)-1))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B83232A5-F125-47B3-9149-56BB9AFFAB52}" name="Tempo Total do Exercício" totalsRowFunction="custom" totalsRowDxfId="0">
+    <tableColumn id="8" xr3:uid="{B83232A5-F125-47B3-9149-56BB9AFFAB52}" name="Tempo Total do Exercício" totalsRowFunction="custom" totalsRowDxfId="12">
       <calculatedColumnFormula array="1">_xlfn.LET(
     _xlpm.cadencia, Tabela1[[#This Row],[Cadência (TUT)]],
     _xlpm.soma_cadencia, SUM(VALUE(_xlfn.TEXTSPLIT(_xlpm.cadencia, "-"))),
@@ -658,30 +634,32 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C248EC49-0D93-48E6-9012-1A316B832A36}" name="Tabela7" displayName="Tabela7" ref="E1:I28" totalsRowCount="1" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C248EC49-0D93-48E6-9012-1A316B832A36}" name="Tabela7" displayName="Tabela7" ref="E1:I28" totalsRowCount="1" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="E1:I27" xr:uid="{C248EC49-0D93-48E6-9012-1A316B832A36}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{1384F953-4707-4BD7-AADD-50B36152BD2A}" name="Métodos/Objetivos" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{1384F953-4707-4BD7-AADD-50B36152BD2A}" name="Métodos/Objetivos" dataDxfId="9">
       <calculatedColumnFormula>Tabela3[[#This Row],[Métodos]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C50B37F1-BBC8-4F9E-9AE0-482AC1CB9284}" name="Hipertrofia" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{ABB978A5-EA43-47A4-8FEC-39EFFDDCED2A}" name="Força Máxima" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{5A014027-31EC-4344-9D19-90473C9720A6}" name="Resistência Muscular" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{92592DA2-E68B-424F-98B2-AB304D4ED6C9}" name="Manutenção/Reabilitação" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{C50B37F1-BBC8-4F9E-9AE0-482AC1CB9284}" name="Hipertrofia" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{ABB978A5-EA43-47A4-8FEC-39EFFDDCED2A}" name="Força Máxima" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{5A014027-31EC-4344-9D19-90473C9720A6}" name="Resistência Muscular" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{92592DA2-E68B-424F-98B2-AB304D4ED6C9}" name="Manutenção/Reabilitação" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{1B705FF1-E851-49A1-859F-5492F0FA3E5A}" name="Tabela8" displayName="Tabela8" ref="K1:O26" totalsRowShown="0">
-  <autoFilter ref="K1:O26" xr:uid="{1B705FF1-E851-49A1-859F-5492F0FA3E5A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{1B705FF1-E851-49A1-859F-5492F0FA3E5A}" name="Tabela8" displayName="Tabela8" ref="K1:O27" totalsRowShown="0">
+  <autoFilter ref="K1:O27" xr:uid="{1B705FF1-E851-49A1-859F-5492F0FA3E5A}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{8D9AF5BD-B494-4F89-9048-A658A8A5ACEA}" name="Métodos/Objetivos"/>
-    <tableColumn id="2" xr3:uid="{6450C433-4BCE-4A0D-BBC9-3CCCFCBEC59F}" name="Hipertrofia" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{10AE9741-AC0B-4111-ABAF-6787051E2871}" name="Força Máxima" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{A465DD72-055A-44EC-9D49-61E696058B10}" name="Resistência Muscular" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{0341FCC7-F940-43C5-AF9D-572D62FDAE20}" name="Manutenção/Reabilitação" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{8D9AF5BD-B494-4F89-9048-A658A8A5ACEA}" name="Métodos/Objetivos" dataDxfId="0">
+      <calculatedColumnFormula>Tabela3[[#This Row],[Métodos]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="2" xr3:uid="{6450C433-4BCE-4A0D-BBC9-3CCCFCBEC59F}" name="Hipertrofia" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{10AE9741-AC0B-4111-ABAF-6787051E2871}" name="Força Máxima" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{A465DD72-055A-44EC-9D49-61E696058B10}" name="Resistência Muscular" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{0341FCC7-F940-43C5-AF9D-572D62FDAE20}" name="Manutenção/Reabilitação" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1006,7 +984,7 @@
         <v>41</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -1042,7 +1020,7 @@
         <v>41</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D3">
         <v>12</v>
@@ -1078,10 +1056,10 @@
         <v>41</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D4">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
         <v>36</v>
@@ -1106,7 +1084,7 @@
     _xlpm.descanso_num, VALUE(SUBSTITUTE(_xlpm.descanso_texto, "s", "")),
     (_xlpm.soma_cadencia * _xlpm.soma_reps * _xlpm.soma_series) + ((_xlpm.soma_series - 1) * _xlpm.descanso_num)
 )/60</f>
-        <v>5.25</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -1114,10 +1092,10 @@
         <v>41</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D5">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
         <v>36</v>
@@ -1142,7 +1120,7 @@
     _xlpm.descanso_num, VALUE(SUBSTITUTE(_xlpm.descanso_texto, "s", "")),
     (_xlpm.soma_cadencia * _xlpm.soma_reps * _xlpm.soma_series) + ((_xlpm.soma_series - 1) * _xlpm.descanso_num)
 )/60</f>
-        <v>5.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1150,10 +1128,10 @@
         <v>41</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D6">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
         <v>36</v>
@@ -1178,7 +1156,7 @@
     _xlpm.descanso_num, VALUE(SUBSTITUTE(_xlpm.descanso_texto, "s", "")),
     (_xlpm.soma_cadencia * _xlpm.soma_reps * _xlpm.soma_series) + ((_xlpm.soma_series - 1) * _xlpm.descanso_num)
 )/60</f>
-        <v>5.75</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -1186,10 +1164,10 @@
         <v>41</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D7">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
         <v>36</v>
@@ -1214,7 +1192,7 @@
     _xlpm.descanso_num, VALUE(SUBSTITUTE(_xlpm.descanso_texto, "s", "")),
     (_xlpm.soma_cadencia * _xlpm.soma_reps * _xlpm.soma_series) + ((_xlpm.soma_series - 1) * _xlpm.descanso_num)
 )/60</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1222,7 +1200,7 @@
         <v>41</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D8">
         <v>12</v>
@@ -1256,7 +1234,7 @@
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H9" s="10">
         <f ca="1">(SUM(Tabela1[Tempo Total do Exercício])/60)/24</f>
-        <v>2.6041666666666668E-2</v>
+        <v>2.4305555555555556E-2</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1264,7 +1242,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B8" xr:uid="{670BF4F2-4951-409E-ACA2-591449D6400A}">
       <formula1>ListaMetodos</formula1>
     </dataValidation>
@@ -1275,7 +1253,7 @@
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B80F030B-DCA7-4B2D-B580-1ED591D0115D}">
           <x14:formula1>
             <xm:f>Dados!$C$2:$C$5</xm:f>
@@ -1368,8 +1346,9 @@
       <c r="I2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="K2" t="s">
-        <v>41</v>
+      <c r="K2" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Default</v>
       </c>
       <c r="L2" s="5">
         <v>60</v>
@@ -1407,8 +1386,9 @@
       <c r="I3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K3" t="s">
-        <v>12</v>
+      <c r="K3" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Drop-set</v>
       </c>
       <c r="L3" s="5">
         <v>120</v>
@@ -1446,8 +1426,9 @@
       <c r="I4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K4" t="s">
-        <v>13</v>
+      <c r="K4" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Rest-Pause</v>
       </c>
       <c r="L4" s="5">
         <v>10</v>
@@ -1485,8 +1466,9 @@
       <c r="I5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K5" t="s">
-        <v>14</v>
+      <c r="K5" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Cluster Sets</v>
       </c>
       <c r="L5" s="5">
         <v>20</v>
@@ -1521,8 +1503,9 @@
       <c r="I6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K6" t="s">
-        <v>15</v>
+      <c r="K6" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Falha Concêntrica</v>
       </c>
       <c r="L6" s="5">
         <v>90</v>
@@ -1557,14 +1540,15 @@
       <c r="I7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K7" t="s">
-        <v>16</v>
+      <c r="K7" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Bi-set</v>
       </c>
       <c r="L7" s="5">
         <v>90</v>
       </c>
       <c r="M7" s="5" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="N7" s="5">
         <v>45</v>
@@ -1593,14 +1577,15 @@
       <c r="I8" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K8" t="s">
-        <v>17</v>
+      <c r="K8" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Tri-set</v>
       </c>
       <c r="L8" s="5">
         <v>120</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="N8" s="5">
         <v>60</v>
@@ -1629,14 +1614,15 @@
       <c r="I9" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K9" t="s">
-        <v>18</v>
+      <c r="K9" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Giant Set</v>
       </c>
       <c r="L9" s="5">
         <v>180</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="N9" s="5">
         <v>90</v>
@@ -1665,8 +1651,9 @@
       <c r="I10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K10" t="s">
-        <v>47</v>
+      <c r="K10" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Supersérie (Antagonista)</v>
       </c>
       <c r="L10" s="5">
         <v>90</v>
@@ -1701,14 +1688,15 @@
       <c r="I11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K11" t="s">
-        <v>48</v>
+      <c r="K11" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Supersérie (Agonista)</v>
       </c>
       <c r="L11" s="5">
         <v>120</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="N11" s="5">
         <v>60</v>
@@ -1732,13 +1720,14 @@
         <v>42</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="K12" t="s">
-        <v>49</v>
+        <v>48</v>
+      </c>
+      <c r="K12" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Tempo sob Tensão (TUT/Cadência)</v>
       </c>
       <c r="L12" s="5">
         <v>90</v>
@@ -1762,19 +1751,20 @@
         <v>Isometria</v>
       </c>
       <c r="F13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="K13" t="s">
-        <v>22</v>
+      <c r="K13" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Isometria</v>
       </c>
       <c r="L13" s="5">
         <v>90</v>
@@ -1809,8 +1799,9 @@
       <c r="I14" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K14" t="s">
-        <v>56</v>
+      <c r="K14" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Repetições Parciais</v>
       </c>
       <c r="L14" s="5">
         <v>60</v>
@@ -1845,8 +1836,9 @@
       <c r="I15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K15" t="s">
-        <v>57</v>
+      <c r="K15" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Pirâmide Crescente</v>
       </c>
       <c r="L15" s="5">
         <v>90</v>
@@ -1881,8 +1873,9 @@
       <c r="I16" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K16" t="s">
-        <v>58</v>
+      <c r="K16" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Pirâmide Decrescente</v>
       </c>
       <c r="L16" s="5">
         <v>90</v>
@@ -1915,10 +1908,11 @@
         <v>44</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="K17" t="s">
-        <v>26</v>
+        <v>47</v>
+      </c>
+      <c r="K17" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Treino em Circuito</v>
       </c>
       <c r="L17" s="5">
         <v>0</v>
@@ -1953,14 +1947,15 @@
       <c r="I18" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K18" t="s">
-        <v>27</v>
+      <c r="K18" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Pré-Exaustão</v>
       </c>
       <c r="L18" s="5">
         <v>90</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="N18" s="5">
         <v>45</v>
@@ -1989,14 +1984,15 @@
       <c r="I19" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K19" t="s">
-        <v>28</v>
+      <c r="K19" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Pós-Exaustão</v>
       </c>
       <c r="L19" s="5">
         <v>90</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="N19" s="5">
         <v>45</v>
@@ -2014,19 +2010,20 @@
         <v>Séries Negativas</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K20" t="s">
-        <v>29</v>
+        <v>54</v>
+      </c>
+      <c r="K20" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Séries Negativas</v>
       </c>
       <c r="L20" s="5">
         <v>120</v>
@@ -2061,8 +2058,9 @@
       <c r="I21" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K21" t="s">
-        <v>62</v>
+      <c r="K21" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Repetições Forçadas</v>
       </c>
       <c r="L21" s="5">
         <v>120</v>
@@ -2097,8 +2095,9 @@
       <c r="I22" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K22" t="s">
-        <v>63</v>
+      <c r="K22" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Repetições Roubadas</v>
       </c>
       <c r="L22" s="5">
         <v>90</v>
@@ -2133,8 +2132,9 @@
       <c r="I23" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K23" t="s">
-        <v>32</v>
+      <c r="K23" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Myo-reps</v>
       </c>
       <c r="L23" s="5">
         <v>15</v>
@@ -2158,19 +2158,20 @@
         <v>Slow Training</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="K24" t="s">
-        <v>33</v>
+        <v>59</v>
+      </c>
+      <c r="K24" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Slow Training</v>
       </c>
       <c r="L24" s="5">
         <v>90</v>
@@ -2205,8 +2206,9 @@
       <c r="I25" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K25" t="s">
-        <v>34</v>
+      <c r="K25" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>Escada (Ladder)</v>
       </c>
       <c r="L25" s="5">
         <v>30</v>
@@ -2223,7 +2225,7 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="E26" s="1" t="str">
         <f>Tabela3[[#This Row],[Métodos]]</f>
@@ -2239,10 +2241,11 @@
         <v>44</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="K26" t="s">
-        <v>68</v>
+        <v>47</v>
+      </c>
+      <c r="K26" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>EMOM (Every Minute on the Minute)</v>
       </c>
       <c r="L26" s="5">
         <v>0</v>
@@ -2259,7 +2262,7 @@
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="E27" s="2" t="str">
         <f>Tabela3[[#This Row],[Métodos]]</f>
@@ -2275,7 +2278,23 @@
         <v>44</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
+      </c>
+      <c r="K27" t="str">
+        <f>Tabela3[[#This Row],[Métodos]]</f>
+        <v>AMRAP (As Many Reps (ou Rounds) As Possible)</v>
+      </c>
+      <c r="L27" s="5">
+        <v>0</v>
+      </c>
+      <c r="M27" s="5">
+        <v>0</v>
+      </c>
+      <c r="N27" s="5">
+        <v>0</v>
+      </c>
+      <c r="O27" s="5">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>